<commit_message>
feat: actualizaciones en leader-streaks, mood-checkins, recognition y widgets
</commit_message>
<xml_diff>
--- a/docs/Plantilla_Onboarding_EvaPro.xlsx
+++ b/docs/Plantilla_Onboarding_EvaPro.xlsx
@@ -1,23 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B57A78E-98BA-491C-AC33-5FC758ADD6EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="1. Organizacion" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="2. Administrador" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="3. Departamentos" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="4. Cargos y Niveles" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="5. Competencias" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="6. Colaboradores" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="Instrucciones" state="visible" r:id="rId10"/>
+    <sheet name="1. Organizacion" sheetId="1" r:id="rId1"/>
+    <sheet name="2. Administrador" sheetId="2" r:id="rId2"/>
+    <sheet name="3. Departamentos" sheetId="3" r:id="rId3"/>
+    <sheet name="4. Cargos y Niveles" sheetId="4" r:id="rId4"/>
+    <sheet name="5. Competencias" sheetId="5" r:id="rId5"/>
+    <sheet name="6. Colaboradores" sheetId="6" r:id="rId6"/>
+    <sheet name="Instrucciones" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="125">
   <si>
     <t>DATOS DE LA ORGANIZACION</t>
   </si>
@@ -386,87 +390,108 @@
   </si>
   <si>
     <t>- tenant_admin = Administrador | manager = Encargado de equipo | employee = Colaborador | external = Asesor externo</t>
+  </si>
+  <si>
+    <t>Nombre representante legal</t>
+  </si>
+  <si>
+    <t>RUT representante legal</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="15" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFC9933A"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF888888"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFC9933A"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF888888"/>
       <sz val="9"/>
+      <color rgb="FF6366F1"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
+      <sz val="14"/>
+      <color rgb="FF6366F1"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="14"/>
+      <color rgb="FF10B981"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF6366F1"/>
-      <sz val="9"/>
+      <sz val="14"/>
+      <color rgb="FFF59E0B"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF6366F1"/>
       <sz val="14"/>
+      <color rgb="FF8B5CF6"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF10B981"/>
       <sz val="14"/>
+      <color rgb="FF38BDF8"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFF59E0B"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF8B5CF6"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF38BDF8"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b/>
+      <sz val="16"/>
       <color rgb="FFC9933A"/>
-      <sz val="16"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="10"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFEF4444"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -476,6 +501,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC9933A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -491,7 +522,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -509,6 +540,9 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -847,21 +881,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="45" customWidth="1"/>
     <col min="3" max="3" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="1" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -944,65 +978,78 @@
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="B11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="B11" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="17" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="B12" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="17" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B13" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="2" t="s">
+      <c r="B13" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="17" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="4"/>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
         <v>25</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="6" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>27</v>
       </c>
@@ -1097,21 +1144,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C24"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="35" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="7" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>6</v>
       </c>
@@ -1352,14 +1399,14 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D19"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="35" customWidth="1"/>
@@ -1367,7 +1414,7 @@
     <col min="4" max="4" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="8" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>6</v>
       </c>
@@ -1601,14 +1648,14 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E19"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -1617,7 +1664,7 @@
     <col min="5" max="5" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="9" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>6</v>
       </c>
@@ -1899,14 +1946,14 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:J54"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="3" width="18" customWidth="1"/>
@@ -1919,7 +1966,7 @@
     <col min="10" max="10" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="10" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>79</v>
       </c>
@@ -3558,59 +3605,59 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:A26"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="95" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" s="11" customFormat="1" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="3" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" s="12" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="4" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" s="12" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="5" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" s="12" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="6" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" s="12" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="7" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" s="12" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="8" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" s="12" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="9" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" s="12" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="10" spans="1:1" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A10" s="13" t="s">
         <v>6</v>
       </c>
@@ -3620,22 +3667,22 @@
         <v>110</v>
       </c>
     </row>
-    <row r="12" spans="1:1" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A12" s="13" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="13" spans="1:1" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A13" s="13" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="14" spans="1:1" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A14" s="13" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="15" spans="1:1" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A15" s="13" t="s">
         <v>6</v>
       </c>
@@ -3645,27 +3692,27 @@
         <v>114</v>
       </c>
     </row>
-    <row r="17" spans="1:1" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A17" s="13" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="18" spans="1:1" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A18" s="13" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="19" spans="1:1" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A19" s="13" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="20" spans="1:1" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A20" s="13" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="21" spans="1:1" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A21" s="13" t="s">
         <v>6</v>
       </c>
@@ -3675,12 +3722,12 @@
         <v>119</v>
       </c>
     </row>
-    <row r="23" spans="1:1" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A23" s="13" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="24" spans="1:1" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A24" s="13" t="s">
         <v>6</v>
       </c>
@@ -3690,13 +3737,13 @@
         <v>121</v>
       </c>
     </row>
-    <row r="26" spans="1:1" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A26" s="13" t="s">
         <v>122</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>